<commit_message>
Enhance candidate detail profile
</commit_message>
<xml_diff>
--- a/template_candidate_data.xlsx
+++ b/template_candidate_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -456,22 +456,26 @@
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="58" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,67 +536,87 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>3년평가</t>
+          <t>2024 평가</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>2025 평가</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>2026 평가</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>리더십</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>어학</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>어학점수</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>어학종류</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>해외경험</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>해외국가</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>해외개월수</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>해외유형</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>자격증</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>주재원적합도</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>팀장적합도</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>후보목적</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>사진URL</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>발령내역</t>
         </is>
       </c>
     </row>
@@ -652,7 +676,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>A, A, A</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -662,49 +686,65 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>890</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>중국 주재</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>24</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>장기 주재</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>품질경영기사</t>
         </is>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>92</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
         <v>87</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>주재원;차기팀장</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2011-03|생산기술팀|사원|입사;2017-01|품질관리팀|대리|전보;2022-01|품질관리팀|과장|승진</t>
         </is>
       </c>
     </row>
@@ -764,7 +804,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>A, A, A</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -774,49 +814,65 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>930</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>인도 파견</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>인도</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>18</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>해외 파견</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>무역영어</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>95</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
         <v>91</v>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>주재원;차기팀장</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2009-06|국내영업팀|사원|입사;2016-03|해외영업팀|과장|전보;2021-01|영업팀|차장|승진</t>
         </is>
       </c>
     </row>
@@ -876,7 +932,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>B+, A, A</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -886,49 +942,65 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>840</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>TOEIC</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>미국 주재</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>30</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>장기 주재</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>기계설계기사</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>86</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Y4" t="n">
         <v>84</v>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>주재원;차기팀장</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2014-07|설계팀|사원|입사;2019-01|선행설계팀|대리|전보;2023-01|설계팀|과장|승진</t>
         </is>
       </c>
     </row>
@@ -943,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1117,192 +1189,240 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>3년평가</t>
+          <t>2024 평가</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>최근 3년 평가 (쉼표로 분리, 예: A, A, A)</t>
+          <t>2024년 평가 등급 (A, B+, B, C, D)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>2025 평가</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2025년 평가 등급 (A, B+, B, C, D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026 평가</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026년 평가 등급 (A, B+, B, C, D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>리더십</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>리더십 평가 (A, B+, B, C, D)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>어학 정보</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>어학</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>어학 시험 종류 (TOEIC, OPIc, IELTS, TEPS, 기타)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>어학점수</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>어학 점수 (숫자만, 예: 890)</t>
-        </is>
-      </c>
+      <c r="B22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>어학</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>어학 시험 종류 (TOEIC, OPIc, IELTS, TEPS, 기타)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>어학점수</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>어학 점수 (숫자만, 예: 890)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>어학종류</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>어학 이름 (예: TOEIC, OPIc IH, IELTS 7.0)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
-      <c r="B24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>해외 경험</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>해외경험</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>해외 경험 유형 (예: 중국 주재, 인도 파견, 미국 출장)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>해외국가</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>국가명 (예: 중국, 인도, 미국)</t>
-        </is>
-      </c>
+      <c r="B27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>해외개월수</t>
+          <t>해외경험</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>해외 경험 개월 수 (숫자만, 예: 24)</t>
+          <t>해외 경험 유형 (예: 중국 주재, 인도 파견, 미국 출장)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>해외국가</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>국가명 (예: 중국, 인도, 미국)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>해외개월수</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>해외 경험 개월 수 (숫자만, 예: 24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>해외유형</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>해외 유형 (장기 주재, 해외 파견, 출장, 단기 파견)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-      <c r="B30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>기타 정보</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>자격증</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>보유 자격증 (예: 품질경영기사, 무역영어)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>주재원적합도</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>주재원 적합도 점수 (1~100, 예: 92)</t>
-        </is>
-      </c>
+      <c r="B33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>팀장적합도</t>
+          <t>자격증</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>차기 팀장 적합도 점수 (1~100, 예: 87)</t>
+          <t>보유 자격증 (예: 품질경영기사, 무역영어)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t>주재원적합도</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>주재원 적합도 점수 (1~100, 예: 92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>팀장적합도</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>차기 팀장 적합도 점수 (1~100, 예: 87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
           <t>후보목적</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>후보 목적 (주재원, 차기팀장, 또는 둘 다 쌍반점으로 분리, 예: 주재원;차기팀장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>사진URL</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>후보자 사진 URL (선택, 예: https://example.com/photo.jpg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>발령내역</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>세미콜론으로 여러 건 입력. 각 건은 날짜|부서|직위|비고 형식 (예: 2022-01|품질관리팀|과장|승진)</t>
         </is>
       </c>
     </row>

</xml_diff>